<commit_message>
Fix meter_rank ordering: restore paper's grouped top-14 convention
The previous commit sorted purely by Test RMSE so rank-1 became `ol-plg`
(a 20-col pair model). When users downloaded the default 10-col
Template_input.xlsx and uploaded only melt comp, the app passed 10
features to a 20-feature pair model → sklearn raised
"X has 10 features, but RandomForestRegressor expects 20" → app crashed
at app.py:228 (the user-reported Step 4 ValueError).

Restore the paper Table 2 / original-meter_rank grouped ordering:
  1-3   liq-* filtered melt-only sheets  (10-col input)
  4-7   single-phase  (ol, cpx, plg, opx)
  8-11  liq-X pairs   (liq-ol, liq-cpx, liq-plg, liq-opx)
  12-14 mineral pairs (ol-cpx, ol-plg, cpx-plg)

Rank-1 is again `melt_only-olpyxspplgsat`, which works out-of-the-box
with the default 10-col template upload. RMSE numbers themselves are
unchanged (still the new 111-exp values).
</commit_message>
<xml_diff>
--- a/meter_rank.xlsx
+++ b/meter_rank.xlsx
@@ -486,29 +486,29 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ol-plg</t>
+          <t>melt_only-olpyxspplgsat</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>497</v>
+        <v>2256</v>
       </c>
       <c r="D2" t="n">
-        <v>0.447</v>
+        <v>0.671</v>
       </c>
       <c r="E2" t="n">
-        <v>1.176</v>
+        <v>1.761</v>
       </c>
       <c r="F2" t="n">
-        <v>15.231</v>
+        <v>18.527</v>
       </c>
       <c r="G2" t="n">
-        <v>39.74</v>
+        <v>48.71</v>
       </c>
       <c r="H2" t="n">
-        <v>0.868</v>
+        <v>1.3</v>
       </c>
       <c r="I2" t="n">
-        <v>2.275</v>
+        <v>3.401</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -522,29 +522,29 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>melt-plg</t>
+          <t>melt_only-pyxspplgsat</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>775</v>
+        <v>1226</v>
       </c>
       <c r="D3" t="n">
-        <v>0.442</v>
+        <v>0.588</v>
       </c>
       <c r="E3" t="n">
-        <v>1.185</v>
+        <v>1.539</v>
       </c>
       <c r="F3" t="n">
-        <v>11.184</v>
+        <v>15.658</v>
       </c>
       <c r="G3" t="n">
-        <v>28.745</v>
+        <v>41.095</v>
       </c>
       <c r="H3" t="n">
-        <v>0.833</v>
+        <v>1.118</v>
       </c>
       <c r="I3" t="n">
-        <v>2.206</v>
+        <v>2.952</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -558,29 +558,29 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>melt-ol</t>
+          <t>melt_only-plgsat</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>765</v>
+        <v>1020</v>
       </c>
       <c r="D4" t="n">
-        <v>0.488</v>
+        <v>0.513</v>
       </c>
       <c r="E4" t="n">
-        <v>1.255</v>
+        <v>1.332</v>
       </c>
       <c r="F4" t="n">
-        <v>14.18</v>
+        <v>12.871</v>
       </c>
       <c r="G4" t="n">
-        <v>37.107</v>
+        <v>34.149</v>
       </c>
       <c r="H4" t="n">
-        <v>0.9340000000000001</v>
+        <v>1.011</v>
       </c>
       <c r="I4" t="n">
-        <v>2.457</v>
+        <v>2.662</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -594,29 +594,29 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>melt_only-plgsat</t>
+          <t>ol_only</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1020</v>
+        <v>776</v>
       </c>
       <c r="D5" t="n">
-        <v>0.513</v>
+        <v>0.661</v>
       </c>
       <c r="E5" t="n">
-        <v>1.332</v>
+        <v>1.752</v>
       </c>
       <c r="F5" t="n">
-        <v>12.871</v>
+        <v>22.348</v>
       </c>
       <c r="G5" t="n">
-        <v>34.149</v>
+        <v>59.266</v>
       </c>
       <c r="H5" t="n">
-        <v>1.011</v>
+        <v>1.204</v>
       </c>
       <c r="I5" t="n">
-        <v>2.662</v>
+        <v>3.223</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -630,29 +630,29 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>melt-cpx</t>
+          <t>cpx_only</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>751</v>
+        <v>766</v>
       </c>
       <c r="D6" t="n">
-        <v>0.547</v>
+        <v>0.713</v>
       </c>
       <c r="E6" t="n">
-        <v>1.434</v>
+        <v>1.858</v>
       </c>
       <c r="F6" t="n">
-        <v>12.996</v>
+        <v>20.261</v>
       </c>
       <c r="G6" t="n">
-        <v>34.411</v>
+        <v>53.728</v>
       </c>
       <c r="H6" t="n">
-        <v>0.799</v>
+        <v>0.828</v>
       </c>
       <c r="I6" t="n">
-        <v>2.084</v>
+        <v>2.247</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -666,29 +666,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ol-cpx</t>
+          <t>plg_only</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>487</v>
+        <v>778</v>
       </c>
       <c r="D7" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.745</v>
       </c>
       <c r="E7" t="n">
-        <v>1.489</v>
+        <v>1.985</v>
       </c>
       <c r="F7" t="n">
-        <v>16.207</v>
+        <v>26.442</v>
       </c>
       <c r="G7" t="n">
-        <v>42.471</v>
+        <v>70.504</v>
       </c>
       <c r="H7" t="n">
-        <v>0.792</v>
+        <v>1.07</v>
       </c>
       <c r="I7" t="n">
-        <v>2.069</v>
+        <v>2.815</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -702,29 +702,29 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>cpx-plg</t>
+          <t>opx_only</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>537</v>
+        <v>287</v>
       </c>
       <c r="D8" t="n">
-        <v>0.573</v>
+        <v>0.765</v>
       </c>
       <c r="E8" t="n">
-        <v>1.526</v>
+        <v>2.007</v>
       </c>
       <c r="F8" t="n">
-        <v>17.857</v>
+        <v>23.414</v>
       </c>
       <c r="G8" t="n">
-        <v>46.832</v>
+        <v>60.947</v>
       </c>
       <c r="H8" t="n">
-        <v>0.605</v>
+        <v>0.885</v>
       </c>
       <c r="I8" t="n">
-        <v>1.611</v>
+        <v>2.261</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -738,29 +738,29 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>melt_only-pyxspplgsat</t>
+          <t>melt-ol</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1226</v>
+        <v>765</v>
       </c>
       <c r="D9" t="n">
-        <v>0.588</v>
+        <v>0.488</v>
       </c>
       <c r="E9" t="n">
-        <v>1.539</v>
+        <v>1.255</v>
       </c>
       <c r="F9" t="n">
-        <v>15.658</v>
+        <v>14.18</v>
       </c>
       <c r="G9" t="n">
-        <v>41.095</v>
+        <v>37.107</v>
       </c>
       <c r="H9" t="n">
-        <v>1.118</v>
+        <v>0.9340000000000001</v>
       </c>
       <c r="I9" t="n">
-        <v>2.952</v>
+        <v>2.457</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -774,29 +774,29 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>melt-opx</t>
+          <t>melt-cpx</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>284</v>
+        <v>751</v>
       </c>
       <c r="D10" t="n">
-        <v>0.619</v>
+        <v>0.547</v>
       </c>
       <c r="E10" t="n">
-        <v>1.626</v>
+        <v>1.434</v>
       </c>
       <c r="F10" t="n">
-        <v>15.73</v>
+        <v>12.996</v>
       </c>
       <c r="G10" t="n">
-        <v>40.592</v>
+        <v>34.411</v>
       </c>
       <c r="H10" t="n">
-        <v>0.794</v>
+        <v>0.799</v>
       </c>
       <c r="I10" t="n">
-        <v>2.009</v>
+        <v>2.084</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -810,29 +810,29 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>melt-sp</t>
+          <t>melt-plg</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>206</v>
+        <v>775</v>
       </c>
       <c r="D11" t="n">
-        <v>0.672</v>
+        <v>0.442</v>
       </c>
       <c r="E11" t="n">
-        <v>1.638</v>
+        <v>1.185</v>
       </c>
       <c r="F11" t="n">
-        <v>19.241</v>
+        <v>11.184</v>
       </c>
       <c r="G11" t="n">
-        <v>50.078</v>
+        <v>28.745</v>
       </c>
       <c r="H11" t="n">
-        <v>1.091</v>
+        <v>0.833</v>
       </c>
       <c r="I11" t="n">
-        <v>2.833</v>
+        <v>2.206</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -846,29 +846,29 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ol_only</t>
+          <t>melt-opx</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>776</v>
+        <v>284</v>
       </c>
       <c r="D12" t="n">
-        <v>0.661</v>
+        <v>0.619</v>
       </c>
       <c r="E12" t="n">
-        <v>1.752</v>
+        <v>1.626</v>
       </c>
       <c r="F12" t="n">
-        <v>22.348</v>
+        <v>15.73</v>
       </c>
       <c r="G12" t="n">
-        <v>59.266</v>
+        <v>40.592</v>
       </c>
       <c r="H12" t="n">
-        <v>1.204</v>
+        <v>0.794</v>
       </c>
       <c r="I12" t="n">
-        <v>3.223</v>
+        <v>2.009</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
@@ -882,29 +882,29 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>melt_only-olpyxspplgsat</t>
+          <t>ol-cpx</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2256</v>
+        <v>487</v>
       </c>
       <c r="D13" t="n">
-        <v>0.671</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="E13" t="n">
-        <v>1.761</v>
+        <v>1.489</v>
       </c>
       <c r="F13" t="n">
-        <v>18.527</v>
+        <v>16.207</v>
       </c>
       <c r="G13" t="n">
-        <v>48.71</v>
+        <v>42.471</v>
       </c>
       <c r="H13" t="n">
-        <v>1.3</v>
+        <v>0.792</v>
       </c>
       <c r="I13" t="n">
-        <v>3.401</v>
+        <v>2.069</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -918,29 +918,29 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>cpx-opx</t>
+          <t>ol-plg</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>215</v>
+        <v>497</v>
       </c>
       <c r="D14" t="n">
-        <v>0.709</v>
+        <v>0.447</v>
       </c>
       <c r="E14" t="n">
-        <v>1.843</v>
+        <v>1.176</v>
       </c>
       <c r="F14" t="n">
-        <v>20.283</v>
+        <v>15.231</v>
       </c>
       <c r="G14" t="n">
-        <v>52.261</v>
+        <v>39.74</v>
       </c>
       <c r="H14" t="n">
-        <v>0.835</v>
+        <v>0.868</v>
       </c>
       <c r="I14" t="n">
-        <v>2.111</v>
+        <v>2.275</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -954,29 +954,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>cpx_only</t>
+          <t>cpx-plg</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>766</v>
+        <v>537</v>
       </c>
       <c r="D15" t="n">
-        <v>0.713</v>
+        <v>0.573</v>
       </c>
       <c r="E15" t="n">
-        <v>1.858</v>
+        <v>1.526</v>
       </c>
       <c r="F15" t="n">
-        <v>20.261</v>
+        <v>17.857</v>
       </c>
       <c r="G15" t="n">
-        <v>53.728</v>
+        <v>46.832</v>
       </c>
       <c r="H15" t="n">
-        <v>0.828</v>
+        <v>0.605</v>
       </c>
       <c r="I15" t="n">
-        <v>2.247</v>
+        <v>1.611</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -985,160 +985,168 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" t="inlineStr">
+      <c r="A16" t="inlineStr"/>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>cpx-opx</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>215</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0.709</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1.843</v>
+      </c>
+      <c r="F17" t="n">
+        <v>20.283</v>
+      </c>
+      <c r="G17" t="n">
+        <v>52.261</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.835</v>
+      </c>
+      <c r="I17" t="n">
+        <v>2.111</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>plg-opx</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="C18" t="n">
         <v>208</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D18" t="n">
         <v>0.721</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E18" t="n">
         <v>1.94</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F18" t="n">
         <v>24.794</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G18" t="n">
         <v>65.69199999999999</v>
       </c>
-      <c r="H16" t="n">
+      <c r="H18" t="n">
         <v>0.799</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I18" t="n">
         <v>1.997</v>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J18" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>plg_only</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>778</v>
-      </c>
-      <c r="D17" t="n">
-        <v>0.745</v>
-      </c>
-      <c r="E17" t="n">
-        <v>1.985</v>
-      </c>
-      <c r="F17" t="n">
-        <v>26.442</v>
-      </c>
-      <c r="G17" t="n">
-        <v>70.504</v>
-      </c>
-      <c r="H17" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="I17" t="n">
-        <v>2.815</v>
-      </c>
-      <c r="J17" t="inlineStr">
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>melt-sp</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>206</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0.672</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1.638</v>
+      </c>
+      <c r="F19" t="n">
+        <v>19.241</v>
+      </c>
+      <c r="G19" t="n">
+        <v>50.078</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1.091</v>
+      </c>
+      <c r="I19" t="n">
+        <v>2.833</v>
+      </c>
+      <c r="J19" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>opx_only</t>
-        </is>
-      </c>
-      <c r="C18" t="n">
-        <v>287</v>
-      </c>
-      <c r="D18" t="n">
-        <v>0.765</v>
-      </c>
-      <c r="E18" t="n">
-        <v>2.007</v>
-      </c>
-      <c r="F18" t="n">
-        <v>23.414</v>
-      </c>
-      <c r="G18" t="n">
-        <v>60.947</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0.885</v>
-      </c>
-      <c r="I18" t="n">
-        <v>2.261</v>
-      </c>
-      <c r="J18" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>sp_only</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>205</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0.825</v>
+      </c>
+      <c r="E20" t="n">
+        <v>2.138</v>
+      </c>
+      <c r="F20" t="n">
+        <v>22.979</v>
+      </c>
+      <c r="G20" t="n">
+        <v>60.449</v>
+      </c>
+      <c r="H20" t="n">
+        <v>1.139</v>
+      </c>
+      <c r="I20" t="n">
+        <v>2.942</v>
+      </c>
+      <c r="J20" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>sp_only</t>
-        </is>
-      </c>
-      <c r="C19" t="n">
-        <v>205</v>
-      </c>
-      <c r="D19" t="n">
-        <v>0.825</v>
-      </c>
-      <c r="E19" t="n">
-        <v>2.138</v>
-      </c>
-      <c r="F19" t="n">
-        <v>22.979</v>
-      </c>
-      <c r="G19" t="n">
-        <v>60.449</v>
-      </c>
-      <c r="H19" t="n">
-        <v>1.139</v>
-      </c>
-      <c r="I19" t="n">
-        <v>2.942</v>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr"/>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1556,29 +1564,29 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>melt-ilm</t>
+          <t>ilm_only</t>
         </is>
       </c>
       <c r="C33" t="n">
         <v>74</v>
       </c>
       <c r="D33" t="n">
-        <v>0.771</v>
+        <v>1.081</v>
       </c>
       <c r="E33" t="n">
-        <v>1.996</v>
+        <v>2.883</v>
       </c>
       <c r="F33" t="n">
-        <v>10.945</v>
+        <v>28.393</v>
       </c>
       <c r="G33" t="n">
-        <v>28.63</v>
+        <v>74.161</v>
       </c>
       <c r="H33" t="n">
-        <v>0.833</v>
+        <v>0.857</v>
       </c>
       <c r="I33" t="n">
-        <v>2.219</v>
+        <v>2.285</v>
       </c>
       <c r="J33" t="inlineStr"/>
     </row>
@@ -1590,29 +1598,29 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ilm_only</t>
+          <t>melt-ilm</t>
         </is>
       </c>
       <c r="C34" t="n">
         <v>74</v>
       </c>
       <c r="D34" t="n">
-        <v>1.081</v>
+        <v>0.771</v>
       </c>
       <c r="E34" t="n">
-        <v>2.883</v>
+        <v>1.996</v>
       </c>
       <c r="F34" t="n">
-        <v>28.393</v>
+        <v>10.945</v>
       </c>
       <c r="G34" t="n">
-        <v>74.161</v>
+        <v>28.63</v>
       </c>
       <c r="H34" t="n">
-        <v>0.857</v>
+        <v>0.833</v>
       </c>
       <c r="I34" t="n">
-        <v>2.285</v>
+        <v>2.219</v>
       </c>
       <c r="J34" t="inlineStr"/>
     </row>
@@ -1692,29 +1700,29 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>opx-mag</t>
+          <t>ol-mag</t>
         </is>
       </c>
       <c r="C37" t="n">
         <v>66</v>
       </c>
       <c r="D37" t="n">
-        <v>0.755</v>
+        <v>0.465</v>
       </c>
       <c r="E37" t="n">
-        <v>1.983</v>
+        <v>1.187</v>
       </c>
       <c r="F37" t="n">
-        <v>18.617</v>
+        <v>12.841</v>
       </c>
       <c r="G37" t="n">
-        <v>45.956</v>
+        <v>33.587</v>
       </c>
       <c r="H37" t="n">
-        <v>0.621</v>
+        <v>1.126</v>
       </c>
       <c r="I37" t="n">
-        <v>1.601</v>
+        <v>2.802</v>
       </c>
       <c r="J37" t="inlineStr"/>
     </row>
@@ -1726,29 +1734,29 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ol-mag</t>
+          <t>opx-mag</t>
         </is>
       </c>
       <c r="C38" t="n">
         <v>66</v>
       </c>
       <c r="D38" t="n">
-        <v>0.465</v>
+        <v>0.755</v>
       </c>
       <c r="E38" t="n">
-        <v>1.187</v>
+        <v>1.983</v>
       </c>
       <c r="F38" t="n">
-        <v>12.841</v>
+        <v>18.617</v>
       </c>
       <c r="G38" t="n">
-        <v>33.587</v>
+        <v>45.956</v>
       </c>
       <c r="H38" t="n">
-        <v>1.126</v>
+        <v>0.621</v>
       </c>
       <c r="I38" t="n">
-        <v>2.802</v>
+        <v>1.601</v>
       </c>
       <c r="J38" t="inlineStr"/>
     </row>
@@ -1862,29 +1870,29 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>melt-grt</t>
+          <t>grt_only</t>
         </is>
       </c>
       <c r="C42" t="n">
         <v>43</v>
       </c>
       <c r="D42" t="n">
-        <v>0.906</v>
+        <v>0.973</v>
       </c>
       <c r="E42" t="n">
-        <v>2.29</v>
+        <v>2.384</v>
       </c>
       <c r="F42" t="n">
-        <v>22.765</v>
+        <v>28.818</v>
       </c>
       <c r="G42" t="n">
-        <v>56.793</v>
+        <v>68.611</v>
       </c>
       <c r="H42" t="n">
-        <v>0.897</v>
+        <v>0.876</v>
       </c>
       <c r="I42" t="n">
-        <v>2.329</v>
+        <v>2.11</v>
       </c>
       <c r="J42" t="inlineStr"/>
     </row>
@@ -1896,29 +1904,29 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>grt_only</t>
+          <t>melt-grt</t>
         </is>
       </c>
       <c r="C43" t="n">
         <v>43</v>
       </c>
       <c r="D43" t="n">
-        <v>0.973</v>
+        <v>0.906</v>
       </c>
       <c r="E43" t="n">
-        <v>2.384</v>
+        <v>2.29</v>
       </c>
       <c r="F43" t="n">
-        <v>28.818</v>
+        <v>22.765</v>
       </c>
       <c r="G43" t="n">
-        <v>68.611</v>
+        <v>56.793</v>
       </c>
       <c r="H43" t="n">
-        <v>0.876</v>
+        <v>0.897</v>
       </c>
       <c r="I43" t="n">
-        <v>2.11</v>
+        <v>2.329</v>
       </c>
       <c r="J43" t="inlineStr"/>
     </row>
@@ -1930,29 +1938,29 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ol-amph</t>
+          <t>amph-ilm</t>
         </is>
       </c>
       <c r="C44" t="n">
         <v>36</v>
       </c>
       <c r="D44" t="n">
-        <v>0.627</v>
+        <v>0.618</v>
       </c>
       <c r="E44" t="n">
-        <v>1.476</v>
+        <v>1.652</v>
       </c>
       <c r="F44" t="n">
-        <v>11.148</v>
+        <v>11.255</v>
       </c>
       <c r="G44" t="n">
-        <v>28.488</v>
+        <v>28.259</v>
       </c>
       <c r="H44" t="n">
-        <v>0.721</v>
+        <v>0.596</v>
       </c>
       <c r="I44" t="n">
-        <v>1.652</v>
+        <v>1.408</v>
       </c>
       <c r="J44" t="inlineStr"/>
     </row>
@@ -1964,29 +1972,29 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>amph-ilm</t>
+          <t>ol-amph</t>
         </is>
       </c>
       <c r="C45" t="n">
         <v>36</v>
       </c>
       <c r="D45" t="n">
-        <v>0.618</v>
+        <v>0.627</v>
       </c>
       <c r="E45" t="n">
+        <v>1.476</v>
+      </c>
+      <c r="F45" t="n">
+        <v>11.148</v>
+      </c>
+      <c r="G45" t="n">
+        <v>28.488</v>
+      </c>
+      <c r="H45" t="n">
+        <v>0.721</v>
+      </c>
+      <c r="I45" t="n">
         <v>1.652</v>
-      </c>
-      <c r="F45" t="n">
-        <v>11.255</v>
-      </c>
-      <c r="G45" t="n">
-        <v>28.259</v>
-      </c>
-      <c r="H45" t="n">
-        <v>0.596</v>
-      </c>
-      <c r="I45" t="n">
-        <v>1.408</v>
       </c>
       <c r="J45" t="inlineStr"/>
     </row>

</xml_diff>